<commit_message>
feat(T3): pegawai CRUD + import Excel + export
- PegawaiForm (react-hook-form + zod) + PegawaiTable (TanStack Table) with sort/pagination, RBAC readOnly for viewer, soft-delete
- CRUD API: GET /api/pegawai (search/filter/pagination), POST create, PUT/DELETE /api/pegawai/[id], GET /api/pangkat
- Template .xlsx generation (exceljs) + GET /api/pegawai/template, parse + validate (NIP 18 digit unique, email valid unique, pangkat FK, jenis enum, dates, kredit)
- Import preview validasi OK/gagal + bulk insert via POST /api/pegawai/import?confirm, ImportDialog UI
- Export rekap Excel/CSV via GET /api/pegawai/export?format
- Regen templates/import-template.xlsx with 18-digit NIPs, vitest alias fix, unit tests for excel & validation

Verifiable: download template -> isi 5 baris -> import preview -> confirm -> tabel update -> export
</commit_message>
<xml_diff>
--- a/templates/import-template.xlsx
+++ b/templates/import-template.xlsx
@@ -37,7 +37,7 @@
     <t>kredit</t>
   </si>
   <si>
-    <t>19800101200001001</t>
+    <t>198001012000010001</t>
   </si>
   <si>
     <t>Contoh Pegawai</t>
@@ -58,7 +58,7 @@
     <t>2020-01-01</t>
   </si>
   <si>
-    <t>19800101200001002</t>
+    <t>198001012000010002</t>
   </si>
   <si>
     <t>Fungsional Muda</t>
@@ -93,14 +93,20 @@
     </font>
     <font>
       <b/>
+      <color rgb="FFFFFFFF"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2563EB"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -117,7 +123,9 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -457,19 +465,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <tabColor rgb="FF2563EB"/>
+  </sheetPr>
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="25" customWidth="1"/>
-    <col min="3" max="3" width="30" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="18" customWidth="1"/>
-    <col min="6" max="7" width="14" customWidth="1"/>
-    <col min="8" max="8" width="10" customWidth="1"/>
+    <col min="1" max="8" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -548,6 +553,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:H1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>